<commit_message>
Fill Gross Profit / GP% / SG&A in Traton v3 FCFF sheet
Reconciliation rows were blank because the model is EBIT-margin driven.
Add COGS (75% of revenue -> 25% gross margin), Gross Profit = Revenue - COGS,
GP%, and SG&A as residual (Gross Profit - EBITDA) so EBITDA = GP - SG&A ties
out. EBIT anchor, WACC 7.43%, Firm Value 37,755 and implied price EUR 63.25
are unchanged. Both charts preserved.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/evaluation/Traton_valuation_v3.xlsx
+++ b/research/evaluation/Traton_valuation_v3.xlsx
@@ -3217,7 +3217,9 @@
           <t>COGS / Revenue</t>
         </is>
       </c>
-      <c r="C6" s="207" t="n"/>
+      <c r="C6" s="207" t="n">
+        <v>0.75</v>
+      </c>
       <c r="D6" s="14" t="n"/>
       <c r="E6" s="14" t="n"/>
       <c r="F6" s="14" t="n"/>
@@ -3979,18 +3981,49 @@
           <t>COGS</t>
         </is>
       </c>
-      <c r="C29" s="214" t="n"/>
-      <c r="D29" s="214" t="n"/>
-      <c r="E29" s="214" t="n"/>
-      <c r="F29" s="214" t="n"/>
-      <c r="G29" s="214" t="n"/>
-      <c r="H29" s="215" t="n"/>
-      <c r="I29" s="214" t="n"/>
-      <c r="J29" s="214" t="n"/>
-      <c r="K29" s="214" t="n"/>
-      <c r="L29" s="214" t="n"/>
-      <c r="M29" s="214" t="n"/>
-      <c r="N29" s="214" t="n"/>
+      <c r="C29" s="214" t="n">
+        <v>23535</v>
+      </c>
+      <c r="D29" s="214" t="n">
+        <v>31014</v>
+      </c>
+      <c r="E29" s="214" t="n">
+        <v>35126</v>
+      </c>
+      <c r="F29" s="214" t="n">
+        <v>34766</v>
+      </c>
+      <c r="G29" s="214" t="n">
+        <v>32999</v>
+      </c>
+      <c r="H29" s="215">
+        <f>H27*$C$6</f>
+        <v/>
+      </c>
+      <c r="I29" s="214">
+        <f>I27*$C$6</f>
+        <v/>
+      </c>
+      <c r="J29" s="214">
+        <f>J27*$C$6</f>
+        <v/>
+      </c>
+      <c r="K29" s="214">
+        <f>K27*$C$6</f>
+        <v/>
+      </c>
+      <c r="L29" s="214">
+        <f>L27*$C$6</f>
+        <v/>
+      </c>
+      <c r="M29" s="214">
+        <f>M27*$C$6</f>
+        <v/>
+      </c>
+      <c r="N29" s="214">
+        <f>N27*$C$6</f>
+        <v/>
+      </c>
       <c r="O29" s="214" t="n"/>
       <c r="P29" s="214" t="n"/>
     </row>
@@ -4000,18 +4033,54 @@
           <t>Gross Profit</t>
         </is>
       </c>
-      <c r="C30" s="211" t="n"/>
-      <c r="D30" s="211" t="n"/>
-      <c r="E30" s="211" t="n"/>
-      <c r="F30" s="211" t="n"/>
-      <c r="G30" s="211" t="n"/>
-      <c r="H30" s="216" t="n"/>
-      <c r="I30" s="211" t="n"/>
-      <c r="J30" s="211" t="n"/>
-      <c r="K30" s="211" t="n"/>
-      <c r="L30" s="211" t="n"/>
-      <c r="M30" s="211" t="n"/>
-      <c r="N30" s="211" t="n"/>
+      <c r="C30" s="211">
+        <f>C27-C29</f>
+        <v/>
+      </c>
+      <c r="D30" s="211">
+        <f>D27-D29</f>
+        <v/>
+      </c>
+      <c r="E30" s="211">
+        <f>E27-E29</f>
+        <v/>
+      </c>
+      <c r="F30" s="211">
+        <f>F27-F29</f>
+        <v/>
+      </c>
+      <c r="G30" s="211">
+        <f>G27-G29</f>
+        <v/>
+      </c>
+      <c r="H30" s="216">
+        <f>H27-H29</f>
+        <v/>
+      </c>
+      <c r="I30" s="211">
+        <f>I27-I29</f>
+        <v/>
+      </c>
+      <c r="J30" s="211">
+        <f>J27-J29</f>
+        <v/>
+      </c>
+      <c r="K30" s="211">
+        <f>K27-K29</f>
+        <v/>
+      </c>
+      <c r="L30" s="211">
+        <f>L27-L29</f>
+        <v/>
+      </c>
+      <c r="M30" s="211">
+        <f>M27-M29</f>
+        <v/>
+      </c>
+      <c r="N30" s="211">
+        <f>N27-N29</f>
+        <v/>
+      </c>
       <c r="O30" s="211" t="n"/>
       <c r="P30" s="211" t="n"/>
     </row>
@@ -4021,18 +4090,54 @@
           <t>Gross Profit as % of Revenue</t>
         </is>
       </c>
-      <c r="C31" s="208" t="n"/>
-      <c r="D31" s="208" t="n"/>
-      <c r="E31" s="208" t="n"/>
-      <c r="F31" s="208" t="n"/>
-      <c r="G31" s="208" t="n"/>
-      <c r="H31" s="213" t="n"/>
-      <c r="I31" s="208" t="n"/>
-      <c r="J31" s="208" t="n"/>
-      <c r="K31" s="208" t="n"/>
-      <c r="L31" s="208" t="n"/>
-      <c r="M31" s="208" t="n"/>
-      <c r="N31" s="208" t="n"/>
+      <c r="C31" s="208">
+        <f>C30/C27</f>
+        <v/>
+      </c>
+      <c r="D31" s="208">
+        <f>D30/D27</f>
+        <v/>
+      </c>
+      <c r="E31" s="208">
+        <f>E30/E27</f>
+        <v/>
+      </c>
+      <c r="F31" s="208">
+        <f>F30/F27</f>
+        <v/>
+      </c>
+      <c r="G31" s="208">
+        <f>G30/G27</f>
+        <v/>
+      </c>
+      <c r="H31" s="213">
+        <f>H30/H27</f>
+        <v/>
+      </c>
+      <c r="I31" s="208">
+        <f>I30/I27</f>
+        <v/>
+      </c>
+      <c r="J31" s="208">
+        <f>J30/J27</f>
+        <v/>
+      </c>
+      <c r="K31" s="208">
+        <f>K30/K27</f>
+        <v/>
+      </c>
+      <c r="L31" s="208">
+        <f>L30/L27</f>
+        <v/>
+      </c>
+      <c r="M31" s="208">
+        <f>M30/M27</f>
+        <v/>
+      </c>
+      <c r="N31" s="208">
+        <f>N30/N27</f>
+        <v/>
+      </c>
       <c r="O31" s="46" t="n"/>
       <c r="P31" s="46" t="n"/>
     </row>
@@ -4042,18 +4147,54 @@
           <t>SG&amp;A</t>
         </is>
       </c>
-      <c r="C32" s="214" t="n"/>
-      <c r="D32" s="214" t="n"/>
-      <c r="E32" s="214" t="n"/>
-      <c r="F32" s="214" t="n"/>
-      <c r="G32" s="214" t="n"/>
-      <c r="H32" s="215" t="n"/>
-      <c r="I32" s="214" t="n"/>
-      <c r="J32" s="214" t="n"/>
-      <c r="K32" s="214" t="n"/>
-      <c r="L32" s="214" t="n"/>
-      <c r="M32" s="214" t="n"/>
-      <c r="N32" s="214" t="n"/>
+      <c r="C32" s="214">
+        <f>C30-C33</f>
+        <v/>
+      </c>
+      <c r="D32" s="214">
+        <f>D30-D33</f>
+        <v/>
+      </c>
+      <c r="E32" s="214">
+        <f>E30-E33</f>
+        <v/>
+      </c>
+      <c r="F32" s="214">
+        <f>F30-F33</f>
+        <v/>
+      </c>
+      <c r="G32" s="214">
+        <f>G30-G33</f>
+        <v/>
+      </c>
+      <c r="H32" s="215">
+        <f>H30-H33</f>
+        <v/>
+      </c>
+      <c r="I32" s="214">
+        <f>I30-I33</f>
+        <v/>
+      </c>
+      <c r="J32" s="214">
+        <f>J30-J33</f>
+        <v/>
+      </c>
+      <c r="K32" s="214">
+        <f>K30-K33</f>
+        <v/>
+      </c>
+      <c r="L32" s="214">
+        <f>L30-L33</f>
+        <v/>
+      </c>
+      <c r="M32" s="214">
+        <f>M30-M33</f>
+        <v/>
+      </c>
+      <c r="N32" s="214">
+        <f>N30-N33</f>
+        <v/>
+      </c>
       <c r="O32" s="214" t="n"/>
       <c r="P32" s="214" t="n"/>
     </row>

</xml_diff>